<commit_message>
Add Shasta County results
</commit_message>
<xml_diff>
--- a/inputs/counties/shasta/detail.xlsx
+++ b/inputs/counties/shasta/detail.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="153">
   <si>
     <t xml:space="preserve">Table of Contents</t>
   </si>
@@ -62,391 +62,409 @@
     <t xml:space="preserve">0120390</t>
   </si>
   <si>
-    <t xml:space="preserve">26.65%</t>
+    <t xml:space="preserve">49.95%</t>
   </si>
   <si>
     <t xml:space="preserve">0120400</t>
   </si>
   <si>
-    <t xml:space="preserve">24.93%</t>
+    <t xml:space="preserve">48.36%</t>
   </si>
   <si>
     <t xml:space="preserve">0120463</t>
   </si>
   <si>
-    <t xml:space="preserve">0.00%</t>
+    <t xml:space="preserve">58.54%</t>
   </si>
   <si>
     <t xml:space="preserve">0120523</t>
   </si>
   <si>
-    <t xml:space="preserve">31.99%</t>
+    <t xml:space="preserve">53.20%</t>
   </si>
   <si>
     <t xml:space="preserve">0120570</t>
   </si>
   <si>
-    <t xml:space="preserve">41.01%</t>
+    <t xml:space="preserve">61.45%</t>
   </si>
   <si>
     <t xml:space="preserve">0120660</t>
   </si>
   <si>
-    <t xml:space="preserve">29.85%</t>
+    <t xml:space="preserve">50.24%</t>
   </si>
   <si>
     <t xml:space="preserve">0120894</t>
   </si>
   <si>
-    <t xml:space="preserve">30.28%</t>
+    <t xml:space="preserve">54.33%</t>
   </si>
   <si>
     <t xml:space="preserve">0120897</t>
   </si>
   <si>
-    <t xml:space="preserve">28.67%</t>
+    <t xml:space="preserve">48.57%</t>
   </si>
   <si>
     <t xml:space="preserve">0121120</t>
   </si>
   <si>
-    <t xml:space="preserve">29.15%</t>
+    <t xml:space="preserve">48.38%</t>
   </si>
   <si>
     <t xml:space="preserve">0121750</t>
   </si>
   <si>
-    <t xml:space="preserve">32.96%</t>
+    <t xml:space="preserve">55.13%</t>
   </si>
   <si>
     <t xml:space="preserve">0190201</t>
   </si>
   <si>
-    <t xml:space="preserve">31.75%</t>
+    <t xml:space="preserve">52.67%</t>
   </si>
   <si>
     <t xml:space="preserve">0220160</t>
   </si>
   <si>
-    <t xml:space="preserve">31.33%</t>
+    <t xml:space="preserve">56.05%</t>
   </si>
   <si>
     <t xml:space="preserve">0220170</t>
   </si>
   <si>
-    <t xml:space="preserve">33.90%</t>
+    <t xml:space="preserve">57.75%</t>
   </si>
   <si>
     <t xml:space="preserve">0220460</t>
   </si>
   <si>
-    <t xml:space="preserve">24.58%</t>
+    <t xml:space="preserve">46.87%</t>
   </si>
   <si>
     <t xml:space="preserve">0220575</t>
   </si>
   <si>
-    <t xml:space="preserve">40.25%</t>
+    <t xml:space="preserve">63.00%</t>
   </si>
   <si>
     <t xml:space="preserve">0220760</t>
   </si>
   <si>
-    <t xml:space="preserve">23.94%</t>
+    <t xml:space="preserve">52.80%</t>
   </si>
   <si>
     <t xml:space="preserve">0220770</t>
   </si>
   <si>
-    <t xml:space="preserve">32.55%</t>
+    <t xml:space="preserve">60.61%</t>
   </si>
   <si>
     <t xml:space="preserve">0221979</t>
   </si>
   <si>
-    <t xml:space="preserve">38.43%</t>
+    <t xml:space="preserve">64.93%</t>
   </si>
   <si>
     <t xml:space="preserve">0221982</t>
   </si>
   <si>
-    <t xml:space="preserve">20.04%</t>
+    <t xml:space="preserve">52.78%</t>
   </si>
   <si>
     <t xml:space="preserve">0290260</t>
   </si>
   <si>
-    <t xml:space="preserve">36.06%</t>
+    <t xml:space="preserve">66.27%</t>
   </si>
   <si>
     <t xml:space="preserve">0290462</t>
   </si>
   <si>
+    <t xml:space="preserve">64.20%</t>
+  </si>
+  <si>
     <t xml:space="preserve">0290530</t>
   </si>
   <si>
-    <t xml:space="preserve">20.53%</t>
+    <t xml:space="preserve">65.30%</t>
   </si>
   <si>
     <t xml:space="preserve">0291130</t>
   </si>
   <si>
+    <t xml:space="preserve">51.61%</t>
+  </si>
+  <si>
     <t xml:space="preserve">0291640</t>
   </si>
   <si>
-    <t xml:space="preserve">37.06%</t>
+    <t xml:space="preserve">58.28%</t>
   </si>
   <si>
     <t xml:space="preserve">0291930</t>
   </si>
   <si>
-    <t xml:space="preserve">31.79%</t>
+    <t xml:space="preserve">65.20%</t>
   </si>
   <si>
     <t xml:space="preserve">0320010</t>
   </si>
   <si>
+    <t xml:space="preserve">62.86%</t>
+  </si>
+  <si>
     <t xml:space="preserve">0320068</t>
   </si>
   <si>
-    <t xml:space="preserve">30.03%</t>
+    <t xml:space="preserve">56.04%</t>
   </si>
   <si>
     <t xml:space="preserve">0320376</t>
   </si>
   <si>
+    <t xml:space="preserve">53.19%</t>
+  </si>
+  <si>
     <t xml:space="preserve">0320420</t>
   </si>
   <si>
-    <t xml:space="preserve">25.68%</t>
+    <t xml:space="preserve">53.07%</t>
   </si>
   <si>
     <t xml:space="preserve">0320978</t>
   </si>
   <si>
-    <t xml:space="preserve">40.62%</t>
+    <t xml:space="preserve">67.86%</t>
   </si>
   <si>
     <t xml:space="preserve">0390070</t>
   </si>
   <si>
-    <t xml:space="preserve">35.93%</t>
+    <t xml:space="preserve">61.86%</t>
   </si>
   <si>
     <t xml:space="preserve">0390102</t>
   </si>
   <si>
-    <t xml:space="preserve">30.34%</t>
+    <t xml:space="preserve">60.92%</t>
   </si>
   <si>
     <t xml:space="preserve">0390321</t>
   </si>
   <si>
-    <t xml:space="preserve">26.29%</t>
+    <t xml:space="preserve">50.29%</t>
   </si>
   <si>
     <t xml:space="preserve">0390470</t>
   </si>
   <si>
-    <t xml:space="preserve">36.67%</t>
+    <t xml:space="preserve">64.49%</t>
   </si>
   <si>
     <t xml:space="preserve">0390560</t>
   </si>
   <si>
-    <t xml:space="preserve">30.90%</t>
+    <t xml:space="preserve">63.08%</t>
   </si>
   <si>
     <t xml:space="preserve">0390590</t>
   </si>
   <si>
-    <t xml:space="preserve">36.36%</t>
+    <t xml:space="preserve">67.70%</t>
   </si>
   <si>
     <t xml:space="preserve">0390600</t>
   </si>
   <si>
-    <t xml:space="preserve">33.22%</t>
+    <t xml:space="preserve">63.15%</t>
   </si>
   <si>
     <t xml:space="preserve">0390610</t>
   </si>
   <si>
-    <t xml:space="preserve">26.78%</t>
+    <t xml:space="preserve">54.10%</t>
   </si>
   <si>
     <t xml:space="preserve">0390611</t>
   </si>
   <si>
-    <t xml:space="preserve">33.96%</t>
+    <t xml:space="preserve">64.94%</t>
   </si>
   <si>
     <t xml:space="preserve">0391210</t>
   </si>
   <si>
-    <t xml:space="preserve">35.31%</t>
+    <t xml:space="preserve">59.94%</t>
   </si>
   <si>
     <t xml:space="preserve">0392113</t>
   </si>
   <si>
-    <t xml:space="preserve">27.19%</t>
+    <t xml:space="preserve">60.20%</t>
   </si>
   <si>
     <t xml:space="preserve">0420370</t>
   </si>
   <si>
-    <t xml:space="preserve">20.95%</t>
+    <t xml:space="preserve">50.41%</t>
   </si>
   <si>
     <t xml:space="preserve">0420375</t>
   </si>
   <si>
-    <t xml:space="preserve">27.00%</t>
+    <t xml:space="preserve">58.37%</t>
   </si>
   <si>
     <t xml:space="preserve">0420861</t>
   </si>
   <si>
-    <t xml:space="preserve">26.84%</t>
+    <t xml:space="preserve">54.62%</t>
   </si>
   <si>
     <t xml:space="preserve">0420912</t>
   </si>
   <si>
-    <t xml:space="preserve">35.35%</t>
+    <t xml:space="preserve">62.82%</t>
   </si>
   <si>
     <t xml:space="preserve">0431003</t>
   </si>
   <si>
-    <t xml:space="preserve">25.21%</t>
+    <t xml:space="preserve">53.36%</t>
   </si>
   <si>
     <t xml:space="preserve">0431004</t>
   </si>
   <si>
-    <t xml:space="preserve">23.89%</t>
+    <t xml:space="preserve">50.59%</t>
   </si>
   <si>
     <t xml:space="preserve">0431005</t>
   </si>
   <si>
-    <t xml:space="preserve">27.57%</t>
+    <t xml:space="preserve">51.83%</t>
   </si>
   <si>
     <t xml:space="preserve">0490091</t>
   </si>
   <si>
-    <t xml:space="preserve">27.34%</t>
+    <t xml:space="preserve">55.62%</t>
   </si>
   <si>
     <t xml:space="preserve">0490101</t>
   </si>
   <si>
-    <t xml:space="preserve">30.94%</t>
+    <t xml:space="preserve">62.06%</t>
   </si>
   <si>
     <t xml:space="preserve">0490270</t>
   </si>
   <si>
+    <t xml:space="preserve">60.00%</t>
+  </si>
+  <si>
     <t xml:space="preserve">0490320</t>
   </si>
   <si>
-    <t xml:space="preserve">25.54%</t>
+    <t xml:space="preserve">59.32%</t>
   </si>
   <si>
     <t xml:space="preserve">0490360</t>
   </si>
   <si>
-    <t xml:space="preserve">30.56%</t>
+    <t xml:space="preserve">59.01%</t>
   </si>
   <si>
     <t xml:space="preserve">0490557</t>
   </si>
   <si>
-    <t xml:space="preserve">26.06%</t>
+    <t xml:space="preserve">55.33%</t>
   </si>
   <si>
     <t xml:space="preserve">0490650</t>
   </si>
   <si>
-    <t xml:space="preserve">32.54%</t>
+    <t xml:space="preserve">66.17%</t>
   </si>
   <si>
     <t xml:space="preserve">0510015</t>
   </si>
   <si>
-    <t xml:space="preserve">29.60%</t>
+    <t xml:space="preserve">49.36%</t>
   </si>
   <si>
     <t xml:space="preserve">0510030</t>
   </si>
   <si>
-    <t xml:space="preserve">21.77%</t>
+    <t xml:space="preserve">46.80%</t>
   </si>
   <si>
     <t xml:space="preserve">0511055</t>
   </si>
   <si>
-    <t xml:space="preserve">23.70%</t>
+    <t xml:space="preserve">46.78%</t>
   </si>
   <si>
     <t xml:space="preserve">0520114</t>
   </si>
   <si>
+    <t xml:space="preserve">80.00%</t>
+  </si>
+  <si>
     <t xml:space="preserve">0590080</t>
   </si>
   <si>
-    <t xml:space="preserve">29.93%</t>
+    <t xml:space="preserve">61.40%</t>
   </si>
   <si>
     <t xml:space="preserve">0590330</t>
   </si>
   <si>
-    <t xml:space="preserve">30.24%</t>
+    <t xml:space="preserve">51.88%</t>
   </si>
   <si>
     <t xml:space="preserve">0590331</t>
   </si>
   <si>
-    <t xml:space="preserve">37.86%</t>
+    <t xml:space="preserve">63.92%</t>
   </si>
   <si>
     <t xml:space="preserve">0590531</t>
   </si>
   <si>
-    <t xml:space="preserve">20.75%</t>
+    <t xml:space="preserve">63.10%</t>
   </si>
   <si>
     <t xml:space="preserve">0590940</t>
   </si>
   <si>
-    <t xml:space="preserve">43.47%</t>
+    <t xml:space="preserve">64.11%</t>
   </si>
   <si>
     <t xml:space="preserve">0590942</t>
   </si>
   <si>
-    <t xml:space="preserve">46.34%</t>
+    <t xml:space="preserve">68.70%</t>
   </si>
   <si>
     <t xml:space="preserve">0591310</t>
   </si>
   <si>
-    <t xml:space="preserve">28.01%</t>
+    <t xml:space="preserve">57.16%</t>
   </si>
   <si>
     <t xml:space="preserve">0591620</t>
   </si>
   <si>
-    <t xml:space="preserve">25.48%</t>
+    <t xml:space="preserve">55.91%</t>
   </si>
   <si>
     <t xml:space="preserve">0592970</t>
   </si>
   <si>
-    <t xml:space="preserve">20.61%</t>
+    <t xml:space="preserve">48.90%</t>
   </si>
   <si>
     <t xml:space="preserve">Total:</t>
@@ -455,7 +473,7 @@
     <t xml:space="preserve">Measure A (Vote For 1)</t>
   </si>
   <si>
-    <t xml:space="preserve">30.27%</t>
+    <t xml:space="preserve">56.49%</t>
   </si>
 </sst>
 </file>
@@ -576,7 +594,7 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>
@@ -614,7 +632,7 @@
         <v>2120</v>
       </c>
       <c r="C2">
-        <v>565</v>
+        <v>1059</v>
       </c>
       <c r="D2" t="s">
         <v>15</v>
@@ -628,7 +646,7 @@
         <v>2258</v>
       </c>
       <c r="C3">
-        <v>563</v>
+        <v>1092</v>
       </c>
       <c r="D3" t="s">
         <v>17</v>
@@ -642,7 +660,7 @@
         <v>41</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
         <v>19</v>
@@ -656,7 +674,7 @@
         <v>2060</v>
       </c>
       <c r="C5">
-        <v>659</v>
+        <v>1096</v>
       </c>
       <c r="D5" t="s">
         <v>21</v>
@@ -670,7 +688,7 @@
         <v>1790</v>
       </c>
       <c r="C6">
-        <v>734</v>
+        <v>1100</v>
       </c>
       <c r="D6" t="s">
         <v>23</v>
@@ -684,7 +702,7 @@
         <v>2482</v>
       </c>
       <c r="C7">
-        <v>741</v>
+        <v>1247</v>
       </c>
       <c r="D7" t="s">
         <v>25</v>
@@ -698,7 +716,7 @@
         <v>2774</v>
       </c>
       <c r="C8">
-        <v>840</v>
+        <v>1507</v>
       </c>
       <c r="D8" t="s">
         <v>27</v>
@@ -712,7 +730,7 @@
         <v>2693</v>
       </c>
       <c r="C9">
-        <v>772</v>
+        <v>1308</v>
       </c>
       <c r="D9" t="s">
         <v>29</v>
@@ -726,7 +744,7 @@
         <v>1664</v>
       </c>
       <c r="C10">
-        <v>485</v>
+        <v>805</v>
       </c>
       <c r="D10" t="s">
         <v>31</v>
@@ -740,7 +758,7 @@
         <v>2224</v>
       </c>
       <c r="C11">
-        <v>733</v>
+        <v>1226</v>
       </c>
       <c r="D11" t="s">
         <v>33</v>
@@ -754,7 +772,7 @@
         <v>1726</v>
       </c>
       <c r="C12">
-        <v>548</v>
+        <v>909</v>
       </c>
       <c r="D12" t="s">
         <v>35</v>
@@ -768,7 +786,7 @@
         <v>1497</v>
       </c>
       <c r="C13">
-        <v>469</v>
+        <v>839</v>
       </c>
       <c r="D13" t="s">
         <v>37</v>
@@ -782,7 +800,7 @@
         <v>2407</v>
       </c>
       <c r="C14">
-        <v>816</v>
+        <v>1390</v>
       </c>
       <c r="D14" t="s">
         <v>39</v>
@@ -796,7 +814,7 @@
         <v>3243</v>
       </c>
       <c r="C15">
-        <v>797</v>
+        <v>1520</v>
       </c>
       <c r="D15" t="s">
         <v>41</v>
@@ -810,7 +828,7 @@
         <v>2435</v>
       </c>
       <c r="C16">
-        <v>980</v>
+        <v>1534</v>
       </c>
       <c r="D16" t="s">
         <v>43</v>
@@ -824,7 +842,7 @@
         <v>2799</v>
       </c>
       <c r="C17">
-        <v>670</v>
+        <v>1478</v>
       </c>
       <c r="D17" t="s">
         <v>45</v>
@@ -838,7 +856,7 @@
         <v>2252</v>
       </c>
       <c r="C18">
-        <v>733</v>
+        <v>1365</v>
       </c>
       <c r="D18" t="s">
         <v>47</v>
@@ -852,7 +870,7 @@
         <v>1366</v>
       </c>
       <c r="C19">
-        <v>525</v>
+        <v>887</v>
       </c>
       <c r="D19" t="s">
         <v>49</v>
@@ -866,7 +884,7 @@
         <v>1906</v>
       </c>
       <c r="C20">
-        <v>382</v>
+        <v>1006</v>
       </c>
       <c r="D20" t="s">
         <v>51</v>
@@ -880,7 +898,7 @@
         <v>2099</v>
       </c>
       <c r="C21">
-        <v>757</v>
+        <v>1391</v>
       </c>
       <c r="D21" t="s">
         <v>53</v>
@@ -894,682 +912,682 @@
         <v>81</v>
       </c>
       <c r="C22">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="D22" t="s">
-        <v>19</v>
+        <v>55</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B23">
         <v>487</v>
       </c>
       <c r="C23">
-        <v>100</v>
+        <v>318</v>
       </c>
       <c r="D23" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B24">
         <v>93</v>
       </c>
       <c r="C24">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="D24" t="s">
-        <v>19</v>
+        <v>59</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B25">
         <v>2253</v>
       </c>
       <c r="C25">
-        <v>835</v>
+        <v>1313</v>
       </c>
       <c r="D25" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B26">
         <v>1428</v>
       </c>
       <c r="C26">
-        <v>454</v>
+        <v>931</v>
       </c>
       <c r="D26" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B27">
         <v>35</v>
       </c>
       <c r="C27">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="D27" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B28">
         <v>2937</v>
       </c>
       <c r="C28">
-        <v>882</v>
+        <v>1646</v>
       </c>
       <c r="D28" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B29">
         <v>2055</v>
       </c>
       <c r="C29">
-        <v>599</v>
+        <v>1093</v>
       </c>
       <c r="D29" t="s">
-        <v>31</v>
+        <v>69</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B30">
         <v>3096</v>
       </c>
       <c r="C30">
-        <v>795</v>
+        <v>1643</v>
       </c>
       <c r="D30" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B31">
         <v>2122</v>
       </c>
       <c r="C31">
-        <v>862</v>
+        <v>1440</v>
       </c>
       <c r="D31" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B32">
         <v>590</v>
       </c>
       <c r="C32">
-        <v>212</v>
+        <v>365</v>
       </c>
       <c r="D32" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B33">
         <v>435</v>
       </c>
       <c r="C33">
-        <v>132</v>
+        <v>265</v>
       </c>
       <c r="D33" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B34">
         <v>696</v>
       </c>
       <c r="C34">
-        <v>183</v>
+        <v>350</v>
       </c>
       <c r="D34" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B35">
         <v>1380</v>
       </c>
       <c r="C35">
-        <v>506</v>
+        <v>890</v>
       </c>
       <c r="D35" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B36">
         <v>3058</v>
       </c>
       <c r="C36">
-        <v>945</v>
+        <v>1929</v>
       </c>
       <c r="D36" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B37">
         <v>1254</v>
       </c>
       <c r="C37">
-        <v>456</v>
+        <v>849</v>
       </c>
       <c r="D37" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B38">
         <v>852</v>
       </c>
       <c r="C38">
-        <v>283</v>
+        <v>538</v>
       </c>
       <c r="D38" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B39">
         <v>366</v>
       </c>
       <c r="C39">
-        <v>98</v>
+        <v>198</v>
       </c>
       <c r="D39" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B40">
         <v>1275</v>
       </c>
       <c r="C40">
-        <v>433</v>
+        <v>828</v>
       </c>
       <c r="D40" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B41">
         <v>2778</v>
       </c>
       <c r="C41">
-        <v>981</v>
+        <v>1665</v>
       </c>
       <c r="D41" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B42">
         <v>809</v>
       </c>
       <c r="C42">
-        <v>220</v>
+        <v>487</v>
       </c>
       <c r="D42" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B43">
         <v>2210</v>
       </c>
       <c r="C43">
-        <v>463</v>
+        <v>1114</v>
       </c>
       <c r="D43" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B44">
         <v>2289</v>
       </c>
       <c r="C44">
-        <v>618</v>
+        <v>1336</v>
       </c>
       <c r="D44" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B45">
         <v>2649</v>
       </c>
       <c r="C45">
-        <v>711</v>
+        <v>1447</v>
       </c>
       <c r="D45" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B46">
         <v>3332</v>
       </c>
       <c r="C46">
-        <v>1178</v>
+        <v>2093</v>
       </c>
       <c r="D46" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B47">
         <v>1979</v>
       </c>
       <c r="C47">
-        <v>499</v>
+        <v>1056</v>
       </c>
       <c r="D47" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B48">
         <v>1708</v>
       </c>
       <c r="C48">
-        <v>408</v>
+        <v>864</v>
       </c>
       <c r="D48" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B49">
         <v>2753</v>
       </c>
       <c r="C49">
-        <v>759</v>
+        <v>1427</v>
       </c>
       <c r="D49" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B50">
         <v>1273</v>
       </c>
       <c r="C50">
-        <v>348</v>
+        <v>708</v>
       </c>
       <c r="D50" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B51">
         <v>1700</v>
       </c>
       <c r="C51">
-        <v>526</v>
+        <v>1055</v>
       </c>
       <c r="D51" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B52">
         <v>5</v>
       </c>
       <c r="C52">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D52" t="s">
-        <v>19</v>
+        <v>115</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="B53">
         <v>1116</v>
       </c>
       <c r="C53">
-        <v>285</v>
+        <v>662</v>
       </c>
       <c r="D53" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B54">
         <v>949</v>
       </c>
       <c r="C54">
-        <v>290</v>
+        <v>560</v>
       </c>
       <c r="D54" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="B55">
         <v>591</v>
       </c>
       <c r="C55">
-        <v>154</v>
+        <v>327</v>
       </c>
       <c r="D55" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="B56">
         <v>1549</v>
       </c>
       <c r="C56">
-        <v>504</v>
+        <v>1025</v>
       </c>
       <c r="D56" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="B57">
         <v>2676</v>
       </c>
       <c r="C57">
-        <v>792</v>
+        <v>1321</v>
       </c>
       <c r="D57" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B58">
         <v>1874</v>
       </c>
       <c r="C58">
-        <v>408</v>
+        <v>877</v>
       </c>
       <c r="D58" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B59">
         <v>1785</v>
       </c>
       <c r="C59">
-        <v>423</v>
+        <v>835</v>
       </c>
       <c r="D59" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B60">
         <v>5</v>
       </c>
       <c r="C60">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D60" t="s">
-        <v>19</v>
+        <v>131</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="B61">
         <v>1811</v>
       </c>
       <c r="C61">
-        <v>542</v>
+        <v>1112</v>
       </c>
       <c r="D61" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="B62">
         <v>2768</v>
       </c>
       <c r="C62">
-        <v>837</v>
+        <v>1436</v>
       </c>
       <c r="D62" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="B63">
         <v>1458</v>
       </c>
       <c r="C63">
-        <v>552</v>
+        <v>932</v>
       </c>
       <c r="D63" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="B64">
         <v>477</v>
       </c>
       <c r="C64">
-        <v>99</v>
+        <v>301</v>
       </c>
       <c r="D64" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="B65">
         <v>2441</v>
       </c>
       <c r="C65">
-        <v>1061</v>
+        <v>1565</v>
       </c>
       <c r="D65" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B66">
         <v>1243</v>
       </c>
       <c r="C66">
-        <v>576</v>
+        <v>854</v>
       </c>
       <c r="D66" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B67">
         <v>2638</v>
       </c>
       <c r="C67">
-        <v>739</v>
+        <v>1508</v>
       </c>
       <c r="D67" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="B68">
         <v>1860</v>
       </c>
       <c r="C68">
-        <v>474</v>
+        <v>1040</v>
       </c>
       <c r="D68" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="B69">
         <v>1640</v>
       </c>
       <c r="C69">
-        <v>338</v>
+        <v>802</v>
       </c>
       <c r="D69" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="B70">
         <v>116695</v>
       </c>
       <c r="C70">
-        <v>35329</v>
+        <v>65917</v>
       </c>
       <c r="D70" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
     </row>
   </sheetData>
@@ -1643,25 +1661,25 @@
         <v>2120</v>
       </c>
       <c r="C4">
-        <v>176</v>
+        <v>346</v>
       </c>
       <c r="D4">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E4">
-        <v>186</v>
+        <v>357</v>
       </c>
       <c r="F4">
-        <v>331</v>
+        <v>643</v>
       </c>
       <c r="G4">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="H4">
-        <v>376</v>
+        <v>696</v>
       </c>
       <c r="I4">
-        <v>562</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="5">
@@ -1672,25 +1690,25 @@
         <v>2258</v>
       </c>
       <c r="C5">
-        <v>202</v>
+        <v>375</v>
       </c>
       <c r="D5">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E5">
-        <v>212</v>
+        <v>388</v>
       </c>
       <c r="F5">
-        <v>298</v>
+        <v>643</v>
       </c>
       <c r="G5">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="H5">
-        <v>350</v>
+        <v>701</v>
       </c>
       <c r="I5">
-        <v>562</v>
+        <v>1089</v>
       </c>
     </row>
     <row r="6">
@@ -1701,25 +1719,25 @@
         <v>41</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="D6">
         <v>0</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="G6">
         <v>0</v>
       </c>
       <c r="H6">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="I6">
-        <v>0</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7">
@@ -1730,25 +1748,25 @@
         <v>2060</v>
       </c>
       <c r="C7">
-        <v>238</v>
+        <v>383</v>
       </c>
       <c r="D7">
         <v>15</v>
       </c>
       <c r="E7">
-        <v>253</v>
+        <v>398</v>
       </c>
       <c r="F7">
-        <v>367</v>
+        <v>645</v>
       </c>
       <c r="G7">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="H7">
-        <v>406</v>
+        <v>698</v>
       </c>
       <c r="I7">
-        <v>659</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="8">
@@ -1759,25 +1777,25 @@
         <v>1790</v>
       </c>
       <c r="C8">
-        <v>275</v>
+        <v>391</v>
       </c>
       <c r="D8">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E8">
-        <v>299</v>
+        <v>416</v>
       </c>
       <c r="F8">
-        <v>355</v>
+        <v>600</v>
       </c>
       <c r="G8">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="H8">
-        <v>434</v>
+        <v>682</v>
       </c>
       <c r="I8">
-        <v>733</v>
+        <v>1098</v>
       </c>
     </row>
     <row r="9">
@@ -1788,25 +1806,25 @@
         <v>2482</v>
       </c>
       <c r="C9">
-        <v>309</v>
+        <v>500</v>
       </c>
       <c r="D9">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="E9">
-        <v>333</v>
+        <v>528</v>
       </c>
       <c r="F9">
-        <v>347</v>
+        <v>656</v>
       </c>
       <c r="G9">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H9">
-        <v>407</v>
+        <v>718</v>
       </c>
       <c r="I9">
-        <v>740</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="10">
@@ -1817,25 +1835,25 @@
         <v>2774</v>
       </c>
       <c r="C10">
-        <v>249</v>
+        <v>466</v>
       </c>
       <c r="D10">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E10">
-        <v>264</v>
+        <v>484</v>
       </c>
       <c r="F10">
-        <v>473</v>
+        <v>912</v>
       </c>
       <c r="G10">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="H10">
-        <v>575</v>
+        <v>1021</v>
       </c>
       <c r="I10">
-        <v>839</v>
+        <v>1505</v>
       </c>
     </row>
     <row r="11">
@@ -1846,25 +1864,25 @@
         <v>2693</v>
       </c>
       <c r="C11">
-        <v>251</v>
+        <v>423</v>
       </c>
       <c r="D11">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E11">
-        <v>270</v>
+        <v>444</v>
       </c>
       <c r="F11">
-        <v>424</v>
+        <v>778</v>
       </c>
       <c r="G11">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="H11">
-        <v>500</v>
+        <v>860</v>
       </c>
       <c r="I11">
-        <v>770</v>
+        <v>1304</v>
       </c>
     </row>
     <row r="12">
@@ -1875,25 +1893,25 @@
         <v>1664</v>
       </c>
       <c r="C12">
-        <v>195</v>
+        <v>306</v>
       </c>
       <c r="D12">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="E12">
-        <v>206</v>
+        <v>327</v>
       </c>
       <c r="F12">
-        <v>251</v>
+        <v>431</v>
       </c>
       <c r="G12">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="H12">
-        <v>279</v>
+        <v>477</v>
       </c>
       <c r="I12">
-        <v>485</v>
+        <v>804</v>
       </c>
     </row>
     <row r="13">
@@ -1904,25 +1922,25 @@
         <v>2224</v>
       </c>
       <c r="C13">
-        <v>345</v>
+        <v>543</v>
       </c>
       <c r="D13">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E13">
-        <v>355</v>
+        <v>557</v>
       </c>
       <c r="F13">
-        <v>336</v>
+        <v>623</v>
       </c>
       <c r="G13">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H13">
-        <v>376</v>
+        <v>667</v>
       </c>
       <c r="I13">
-        <v>731</v>
+        <v>1224</v>
       </c>
     </row>
     <row r="14">
@@ -1933,25 +1951,25 @@
         <v>1726</v>
       </c>
       <c r="C14">
-        <v>117</v>
+        <v>213</v>
       </c>
       <c r="D14">
         <v>12</v>
       </c>
       <c r="E14">
-        <v>129</v>
+        <v>225</v>
       </c>
       <c r="F14">
-        <v>309</v>
+        <v>574</v>
       </c>
       <c r="G14">
         <v>110</v>
       </c>
       <c r="H14">
-        <v>419</v>
+        <v>684</v>
       </c>
       <c r="I14">
-        <v>548</v>
+        <v>909</v>
       </c>
     </row>
     <row r="15">
@@ -1962,25 +1980,25 @@
         <v>1497</v>
       </c>
       <c r="C15">
-        <v>152</v>
+        <v>259</v>
       </c>
       <c r="D15">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E15">
-        <v>169</v>
+        <v>278</v>
       </c>
       <c r="F15">
-        <v>232</v>
+        <v>487</v>
       </c>
       <c r="G15">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="H15">
-        <v>297</v>
+        <v>554</v>
       </c>
       <c r="I15">
-        <v>466</v>
+        <v>832</v>
       </c>
     </row>
     <row r="16">
@@ -1991,25 +2009,25 @@
         <v>2407</v>
       </c>
       <c r="C16">
-        <v>253</v>
+        <v>392</v>
       </c>
       <c r="D16">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E16">
-        <v>270</v>
+        <v>413</v>
       </c>
       <c r="F16">
-        <v>453</v>
+        <v>880</v>
       </c>
       <c r="G16">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="H16">
-        <v>544</v>
+        <v>975</v>
       </c>
       <c r="I16">
-        <v>814</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="17">
@@ -2020,25 +2038,25 @@
         <v>3243</v>
       </c>
       <c r="C17">
-        <v>231</v>
+        <v>471</v>
       </c>
       <c r="D17">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E17">
-        <v>261</v>
+        <v>503</v>
       </c>
       <c r="F17">
-        <v>402</v>
+        <v>870</v>
       </c>
       <c r="G17">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="H17">
-        <v>535</v>
+        <v>1016</v>
       </c>
       <c r="I17">
-        <v>796</v>
+        <v>1519</v>
       </c>
     </row>
     <row r="18">
@@ -2049,25 +2067,25 @@
         <v>2435</v>
       </c>
       <c r="C18">
-        <v>364</v>
+        <v>551</v>
       </c>
       <c r="D18">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E18">
-        <v>393</v>
+        <v>582</v>
       </c>
       <c r="F18">
-        <v>501</v>
+        <v>865</v>
       </c>
       <c r="G18">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H18">
-        <v>580</v>
+        <v>945</v>
       </c>
       <c r="I18">
-        <v>973</v>
+        <v>1527</v>
       </c>
     </row>
     <row r="19">
@@ -2078,25 +2096,25 @@
         <v>2799</v>
       </c>
       <c r="C19">
-        <v>270</v>
+        <v>587</v>
       </c>
       <c r="D19">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E19">
-        <v>277</v>
+        <v>597</v>
       </c>
       <c r="F19">
-        <v>350</v>
+        <v>831</v>
       </c>
       <c r="G19">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="H19">
-        <v>392</v>
+        <v>880</v>
       </c>
       <c r="I19">
-        <v>669</v>
+        <v>1477</v>
       </c>
     </row>
     <row r="20">
@@ -2107,25 +2125,25 @@
         <v>2252</v>
       </c>
       <c r="C20">
-        <v>254</v>
+        <v>445</v>
       </c>
       <c r="D20">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E20">
-        <v>270</v>
+        <v>462</v>
       </c>
       <c r="F20">
-        <v>412</v>
+        <v>847</v>
       </c>
       <c r="G20">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="H20">
-        <v>460</v>
+        <v>898</v>
       </c>
       <c r="I20">
-        <v>730</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="21">
@@ -2136,25 +2154,25 @@
         <v>1366</v>
       </c>
       <c r="C21">
-        <v>154</v>
+        <v>243</v>
       </c>
       <c r="D21">
         <v>0</v>
       </c>
       <c r="E21">
-        <v>154</v>
+        <v>243</v>
       </c>
       <c r="F21">
-        <v>331</v>
+        <v>603</v>
       </c>
       <c r="G21">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H21">
-        <v>368</v>
+        <v>641</v>
       </c>
       <c r="I21">
-        <v>522</v>
+        <v>884</v>
       </c>
     </row>
     <row r="22">
@@ -2165,25 +2183,25 @@
         <v>1906</v>
       </c>
       <c r="C22">
-        <v>122</v>
+        <v>313</v>
       </c>
       <c r="D22">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="E22">
-        <v>124</v>
+        <v>325</v>
       </c>
       <c r="F22">
-        <v>249</v>
+        <v>647</v>
       </c>
       <c r="G22">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="H22">
-        <v>258</v>
+        <v>679</v>
       </c>
       <c r="I22">
-        <v>382</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="23">
@@ -2194,25 +2212,25 @@
         <v>2099</v>
       </c>
       <c r="C23">
-        <v>219</v>
+        <v>377</v>
       </c>
       <c r="D23">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E23">
-        <v>234</v>
+        <v>394</v>
       </c>
       <c r="F23">
-        <v>427</v>
+        <v>899</v>
       </c>
       <c r="G23">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H23">
-        <v>522</v>
+        <v>996</v>
       </c>
       <c r="I23">
-        <v>756</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="24">
@@ -2223,871 +2241,871 @@
         <v>81</v>
       </c>
       <c r="C24">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="D24">
         <v>0</v>
       </c>
       <c r="E24">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="F24">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="G24">
         <v>0</v>
       </c>
       <c r="H24">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="I24">
-        <v>0</v>
+        <v>52</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B25">
         <v>487</v>
       </c>
       <c r="C25">
-        <v>29</v>
+        <v>91</v>
       </c>
       <c r="D25">
         <v>4</v>
       </c>
       <c r="E25">
-        <v>33</v>
+        <v>95</v>
       </c>
       <c r="F25">
-        <v>43</v>
+        <v>198</v>
       </c>
       <c r="G25">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H25">
-        <v>67</v>
+        <v>223</v>
       </c>
       <c r="I25">
-        <v>100</v>
+        <v>318</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B26">
         <v>93</v>
       </c>
       <c r="C26">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D26">
         <v>0</v>
       </c>
       <c r="E26">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F26">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="G26">
         <v>0</v>
       </c>
       <c r="H26">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="I26">
-        <v>0</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B27">
         <v>2253</v>
       </c>
       <c r="C27">
-        <v>161</v>
+        <v>261</v>
       </c>
       <c r="D27">
         <v>24</v>
       </c>
       <c r="E27">
-        <v>185</v>
+        <v>285</v>
       </c>
       <c r="F27">
-        <v>481</v>
+        <v>853</v>
       </c>
       <c r="G27">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="H27">
-        <v>650</v>
+        <v>1028</v>
       </c>
       <c r="I27">
-        <v>835</v>
+        <v>1313</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B28">
         <v>1428</v>
       </c>
       <c r="C28">
-        <v>154</v>
+        <v>302</v>
       </c>
       <c r="D28">
         <v>15</v>
       </c>
       <c r="E28">
-        <v>169</v>
+        <v>317</v>
       </c>
       <c r="F28">
-        <v>232</v>
+        <v>556</v>
       </c>
       <c r="G28">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="H28">
-        <v>285</v>
+        <v>614</v>
       </c>
       <c r="I28">
-        <v>454</v>
+        <v>931</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B29">
         <v>35</v>
       </c>
       <c r="C29">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D29">
         <v>0</v>
       </c>
       <c r="E29">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F29">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="G29">
         <v>0</v>
       </c>
       <c r="H29">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="I29">
-        <v>0</v>
+        <v>22</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B30">
         <v>2937</v>
       </c>
       <c r="C30">
-        <v>247</v>
+        <v>484</v>
       </c>
       <c r="D30">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E30">
-        <v>262</v>
+        <v>502</v>
       </c>
       <c r="F30">
-        <v>519</v>
+        <v>1036</v>
       </c>
       <c r="G30">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="H30">
-        <v>618</v>
+        <v>1139</v>
       </c>
       <c r="I30">
-        <v>880</v>
+        <v>1641</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B31">
         <v>2055</v>
       </c>
       <c r="C31">
-        <v>161</v>
+        <v>285</v>
       </c>
       <c r="D31">
         <v>14</v>
       </c>
       <c r="E31">
-        <v>175</v>
+        <v>299</v>
       </c>
       <c r="F31">
-        <v>341</v>
+        <v>707</v>
       </c>
       <c r="G31">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="H31">
-        <v>424</v>
+        <v>792</v>
       </c>
       <c r="I31">
-        <v>599</v>
+        <v>1091</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B32">
         <v>3096</v>
       </c>
       <c r="C32">
-        <v>222</v>
+        <v>467</v>
       </c>
       <c r="D32">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="E32">
-        <v>248</v>
+        <v>497</v>
       </c>
       <c r="F32">
-        <v>443</v>
+        <v>1034</v>
       </c>
       <c r="G32">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="H32">
-        <v>547</v>
+        <v>1146</v>
       </c>
       <c r="I32">
-        <v>795</v>
+        <v>1643</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B33">
         <v>2122</v>
       </c>
       <c r="C33">
-        <v>238</v>
+        <v>383</v>
       </c>
       <c r="D33">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E33">
-        <v>255</v>
+        <v>402</v>
       </c>
       <c r="F33">
-        <v>501</v>
+        <v>927</v>
       </c>
       <c r="G33">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="H33">
-        <v>606</v>
+        <v>1036</v>
       </c>
       <c r="I33">
-        <v>861</v>
+        <v>1438</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B34">
         <v>590</v>
       </c>
       <c r="C34">
-        <v>56</v>
+        <v>85</v>
       </c>
       <c r="D34">
         <v>10</v>
       </c>
       <c r="E34">
-        <v>66</v>
+        <v>95</v>
       </c>
       <c r="F34">
-        <v>101</v>
+        <v>224</v>
       </c>
       <c r="G34">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H34">
-        <v>146</v>
+        <v>270</v>
       </c>
       <c r="I34">
-        <v>212</v>
+        <v>365</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B35">
         <v>435</v>
       </c>
       <c r="C35">
-        <v>13</v>
+        <v>42</v>
       </c>
       <c r="D35">
         <v>5</v>
       </c>
       <c r="E35">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="F35">
-        <v>87</v>
+        <v>188</v>
       </c>
       <c r="G35">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="H35">
-        <v>114</v>
+        <v>218</v>
       </c>
       <c r="I35">
-        <v>132</v>
+        <v>265</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B36">
         <v>696</v>
       </c>
       <c r="C36">
-        <v>34</v>
+        <v>68</v>
       </c>
       <c r="D36">
         <v>2</v>
       </c>
       <c r="E36">
-        <v>36</v>
+        <v>70</v>
       </c>
       <c r="F36">
-        <v>114</v>
+        <v>246</v>
       </c>
       <c r="G36">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H36">
-        <v>147</v>
+        <v>280</v>
       </c>
       <c r="I36">
-        <v>183</v>
+        <v>350</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B37">
         <v>1380</v>
       </c>
       <c r="C37">
-        <v>97</v>
+        <v>169</v>
       </c>
       <c r="D37">
         <v>14</v>
       </c>
       <c r="E37">
-        <v>111</v>
+        <v>183</v>
       </c>
       <c r="F37">
-        <v>301</v>
+        <v>608</v>
       </c>
       <c r="G37">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="H37">
-        <v>393</v>
+        <v>704</v>
       </c>
       <c r="I37">
-        <v>504</v>
+        <v>887</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B38">
         <v>3058</v>
       </c>
       <c r="C38">
-        <v>183</v>
+        <v>369</v>
       </c>
       <c r="D38">
         <v>18</v>
       </c>
       <c r="E38">
-        <v>201</v>
+        <v>387</v>
       </c>
       <c r="F38">
-        <v>585</v>
+        <v>1374</v>
       </c>
       <c r="G38">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="H38">
-        <v>744</v>
+        <v>1541</v>
       </c>
       <c r="I38">
-        <v>945</v>
+        <v>1928</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B39">
         <v>1254</v>
       </c>
       <c r="C39">
-        <v>76</v>
+        <v>139</v>
       </c>
       <c r="D39">
         <v>12</v>
       </c>
       <c r="E39">
-        <v>88</v>
+        <v>151</v>
       </c>
       <c r="F39">
-        <v>250</v>
+        <v>576</v>
       </c>
       <c r="G39">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="H39">
-        <v>368</v>
+        <v>697</v>
       </c>
       <c r="I39">
-        <v>456</v>
+        <v>848</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B40">
         <v>852</v>
       </c>
       <c r="C40">
-        <v>95</v>
+        <v>178</v>
       </c>
       <c r="D40">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E40">
-        <v>105</v>
+        <v>192</v>
       </c>
       <c r="F40">
-        <v>135</v>
+        <v>297</v>
       </c>
       <c r="G40">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="H40">
-        <v>178</v>
+        <v>346</v>
       </c>
       <c r="I40">
-        <v>283</v>
+        <v>538</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B41">
         <v>366</v>
       </c>
       <c r="C41">
-        <v>41</v>
+        <v>70</v>
       </c>
       <c r="D41">
         <v>7</v>
       </c>
       <c r="E41">
-        <v>48</v>
+        <v>77</v>
       </c>
       <c r="F41">
-        <v>34</v>
+        <v>105</v>
       </c>
       <c r="G41">
         <v>16</v>
       </c>
       <c r="H41">
-        <v>50</v>
+        <v>121</v>
       </c>
       <c r="I41">
-        <v>98</v>
+        <v>198</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B42">
         <v>1275</v>
       </c>
       <c r="C42">
-        <v>115</v>
+        <v>194</v>
       </c>
       <c r="D42">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E42">
-        <v>122</v>
+        <v>203</v>
       </c>
       <c r="F42">
-        <v>236</v>
+        <v>550</v>
       </c>
       <c r="G42">
         <v>75</v>
       </c>
       <c r="H42">
-        <v>311</v>
+        <v>625</v>
       </c>
       <c r="I42">
-        <v>433</v>
+        <v>828</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B43">
         <v>2778</v>
       </c>
       <c r="C43">
-        <v>217</v>
+        <v>349</v>
       </c>
       <c r="D43">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="E43">
-        <v>254</v>
+        <v>392</v>
       </c>
       <c r="F43">
-        <v>515</v>
+        <v>1045</v>
       </c>
       <c r="G43">
-        <v>211</v>
+        <v>225</v>
       </c>
       <c r="H43">
-        <v>726</v>
+        <v>1270</v>
       </c>
       <c r="I43">
-        <v>980</v>
+        <v>1662</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B44">
         <v>809</v>
       </c>
       <c r="C44">
-        <v>42</v>
+        <v>82</v>
       </c>
       <c r="D44">
         <v>9</v>
       </c>
       <c r="E44">
-        <v>51</v>
+        <v>91</v>
       </c>
       <c r="F44">
-        <v>134</v>
+        <v>355</v>
       </c>
       <c r="G44">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="H44">
-        <v>168</v>
+        <v>394</v>
       </c>
       <c r="I44">
-        <v>219</v>
+        <v>485</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B45">
         <v>2210</v>
       </c>
       <c r="C45">
-        <v>167</v>
+        <v>386</v>
       </c>
       <c r="D45">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E45">
-        <v>177</v>
+        <v>397</v>
       </c>
       <c r="F45">
-        <v>226</v>
+        <v>650</v>
       </c>
       <c r="G45">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H45">
-        <v>286</v>
+        <v>716</v>
       </c>
       <c r="I45">
-        <v>463</v>
+        <v>1113</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B46">
         <v>2289</v>
       </c>
       <c r="C46">
-        <v>186</v>
+        <v>423</v>
       </c>
       <c r="D46">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E46">
-        <v>199</v>
+        <v>438</v>
       </c>
       <c r="F46">
-        <v>357</v>
+        <v>829</v>
       </c>
       <c r="G46">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="H46">
-        <v>418</v>
+        <v>896</v>
       </c>
       <c r="I46">
-        <v>617</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B47">
         <v>2649</v>
       </c>
       <c r="C47">
-        <v>186</v>
+        <v>428</v>
       </c>
       <c r="D47">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="E47">
-        <v>216</v>
+        <v>462</v>
       </c>
       <c r="F47">
-        <v>359</v>
+        <v>845</v>
       </c>
       <c r="G47">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="H47">
-        <v>495</v>
+        <v>984</v>
       </c>
       <c r="I47">
-        <v>711</v>
+        <v>1446</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B48">
         <v>3332</v>
       </c>
       <c r="C48">
-        <v>308</v>
+        <v>519</v>
       </c>
       <c r="D48">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E48">
-        <v>326</v>
+        <v>539</v>
       </c>
       <c r="F48">
-        <v>686</v>
+        <v>1372</v>
       </c>
       <c r="G48">
-        <v>164</v>
+        <v>177</v>
       </c>
       <c r="H48">
-        <v>850</v>
+        <v>1549</v>
       </c>
       <c r="I48">
-        <v>1176</v>
+        <v>2088</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B49">
         <v>1979</v>
       </c>
       <c r="C49">
-        <v>138</v>
+        <v>309</v>
       </c>
       <c r="D49">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E49">
-        <v>156</v>
+        <v>330</v>
       </c>
       <c r="F49">
-        <v>255</v>
+        <v>637</v>
       </c>
       <c r="G49">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H49">
-        <v>343</v>
+        <v>726</v>
       </c>
       <c r="I49">
-        <v>499</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B50">
         <v>1708</v>
       </c>
       <c r="C50">
-        <v>111</v>
+        <v>235</v>
       </c>
       <c r="D50">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E50">
-        <v>131</v>
+        <v>257</v>
       </c>
       <c r="F50">
-        <v>190</v>
+        <v>514</v>
       </c>
       <c r="G50">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="H50">
-        <v>277</v>
+        <v>606</v>
       </c>
       <c r="I50">
-        <v>408</v>
+        <v>863</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B51">
         <v>2753</v>
       </c>
       <c r="C51">
-        <v>212</v>
+        <v>419</v>
       </c>
       <c r="D51">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E51">
-        <v>244</v>
+        <v>452</v>
       </c>
       <c r="F51">
-        <v>387</v>
+        <v>841</v>
       </c>
       <c r="G51">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="H51">
-        <v>515</v>
+        <v>975</v>
       </c>
       <c r="I51">
-        <v>759</v>
+        <v>1427</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B52">
         <v>1273</v>
       </c>
       <c r="C52">
-        <v>84</v>
+        <v>163</v>
       </c>
       <c r="D52">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E52">
-        <v>97</v>
+        <v>177</v>
       </c>
       <c r="F52">
-        <v>179</v>
+        <v>458</v>
       </c>
       <c r="G52">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H52">
-        <v>250</v>
+        <v>530</v>
       </c>
       <c r="I52">
-        <v>347</v>
+        <v>707</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B53">
         <v>1700</v>
       </c>
       <c r="C53">
-        <v>107</v>
+        <v>194</v>
       </c>
       <c r="D53">
         <v>20</v>
       </c>
       <c r="E53">
-        <v>127</v>
+        <v>214</v>
       </c>
       <c r="F53">
-        <v>279</v>
+        <v>704</v>
       </c>
       <c r="G53">
-        <v>120</v>
+        <v>136</v>
       </c>
       <c r="H53">
-        <v>399</v>
+        <v>840</v>
       </c>
       <c r="I53">
-        <v>526</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B54">
         <v>5</v>
@@ -3102,224 +3120,224 @@
         <v>0</v>
       </c>
       <c r="F54">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G54">
         <v>0</v>
       </c>
       <c r="H54">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I54">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="B55">
         <v>1116</v>
       </c>
       <c r="C55">
-        <v>62</v>
+        <v>133</v>
       </c>
       <c r="D55">
         <v>2</v>
       </c>
       <c r="E55">
-        <v>64</v>
+        <v>135</v>
       </c>
       <c r="F55">
-        <v>159</v>
+        <v>462</v>
       </c>
       <c r="G55">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H55">
-        <v>221</v>
+        <v>527</v>
       </c>
       <c r="I55">
-        <v>285</v>
+        <v>662</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B56">
         <v>949</v>
       </c>
       <c r="C56">
-        <v>79</v>
+        <v>168</v>
       </c>
       <c r="D56">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E56">
-        <v>89</v>
+        <v>181</v>
       </c>
       <c r="F56">
-        <v>145</v>
+        <v>317</v>
       </c>
       <c r="G56">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="H56">
-        <v>201</v>
+        <v>379</v>
       </c>
       <c r="I56">
-        <v>290</v>
+        <v>560</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="B57">
         <v>591</v>
       </c>
       <c r="C57">
-        <v>43</v>
+        <v>86</v>
       </c>
       <c r="D57">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E57">
-        <v>49</v>
+        <v>93</v>
       </c>
       <c r="F57">
-        <v>89</v>
+        <v>214</v>
       </c>
       <c r="G57">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="H57">
-        <v>105</v>
+        <v>233</v>
       </c>
       <c r="I57">
-        <v>154</v>
+        <v>326</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="B58">
         <v>1549</v>
       </c>
       <c r="C58">
-        <v>108</v>
+        <v>215</v>
       </c>
       <c r="D58">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E58">
-        <v>114</v>
+        <v>222</v>
       </c>
       <c r="F58">
-        <v>323</v>
+        <v>730</v>
       </c>
       <c r="G58">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="H58">
-        <v>390</v>
+        <v>803</v>
       </c>
       <c r="I58">
-        <v>504</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="B59">
         <v>2676</v>
       </c>
       <c r="C59">
-        <v>207</v>
+        <v>330</v>
       </c>
       <c r="D59">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E59">
-        <v>230</v>
+        <v>355</v>
       </c>
       <c r="F59">
-        <v>439</v>
+        <v>833</v>
       </c>
       <c r="G59">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="H59">
-        <v>562</v>
+        <v>965</v>
       </c>
       <c r="I59">
-        <v>792</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B60">
         <v>1874</v>
       </c>
       <c r="C60">
-        <v>118</v>
+        <v>227</v>
       </c>
       <c r="D60">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="E60">
-        <v>133</v>
+        <v>249</v>
       </c>
       <c r="F60">
-        <v>208</v>
+        <v>553</v>
       </c>
       <c r="G60">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="H60">
-        <v>275</v>
+        <v>628</v>
       </c>
       <c r="I60">
-        <v>408</v>
+        <v>877</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B61">
         <v>1785</v>
       </c>
       <c r="C61">
-        <v>119</v>
+        <v>254</v>
       </c>
       <c r="D61">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E61">
-        <v>122</v>
+        <v>261</v>
       </c>
       <c r="F61">
-        <v>254</v>
+        <v>524</v>
       </c>
       <c r="G61">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="H61">
-        <v>301</v>
+        <v>574</v>
       </c>
       <c r="I61">
-        <v>423</v>
+        <v>835</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B62">
         <v>5</v>
@@ -3334,306 +3352,306 @@
         <v>0</v>
       </c>
       <c r="F62">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G62">
         <v>0</v>
       </c>
       <c r="H62">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I62">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="B63">
         <v>1811</v>
       </c>
       <c r="C63">
-        <v>95</v>
+        <v>217</v>
       </c>
       <c r="D63">
         <v>14</v>
       </c>
       <c r="E63">
-        <v>109</v>
+        <v>231</v>
       </c>
       <c r="F63">
-        <v>327</v>
+        <v>770</v>
       </c>
       <c r="G63">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="H63">
-        <v>432</v>
+        <v>880</v>
       </c>
       <c r="I63">
-        <v>541</v>
+        <v>1111</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="B64">
         <v>2768</v>
       </c>
       <c r="C64">
-        <v>158</v>
+        <v>277</v>
       </c>
       <c r="D64">
         <v>22</v>
       </c>
       <c r="E64">
-        <v>180</v>
+        <v>299</v>
       </c>
       <c r="F64">
-        <v>543</v>
+        <v>1014</v>
       </c>
       <c r="G64">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H64">
-        <v>657</v>
+        <v>1136</v>
       </c>
       <c r="I64">
-        <v>837</v>
+        <v>1435</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="B65">
         <v>1458</v>
       </c>
       <c r="C65">
-        <v>94</v>
+        <v>144</v>
       </c>
       <c r="D65">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E65">
-        <v>102</v>
+        <v>154</v>
       </c>
       <c r="F65">
-        <v>382</v>
+        <v>695</v>
       </c>
       <c r="G65">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="H65">
-        <v>450</v>
+        <v>777</v>
       </c>
       <c r="I65">
-        <v>552</v>
+        <v>931</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="B66">
         <v>477</v>
       </c>
       <c r="C66">
-        <v>25</v>
+        <v>75</v>
       </c>
       <c r="D66">
         <v>2</v>
       </c>
       <c r="E66">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="F66">
-        <v>56</v>
+        <v>207</v>
       </c>
       <c r="G66">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H66">
-        <v>72</v>
+        <v>224</v>
       </c>
       <c r="I66">
-        <v>99</v>
+        <v>301</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="B67">
         <v>2441</v>
       </c>
       <c r="C67">
-        <v>245</v>
+        <v>388</v>
       </c>
       <c r="D67">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E67">
-        <v>267</v>
+        <v>411</v>
       </c>
       <c r="F67">
-        <v>655</v>
+        <v>1010</v>
       </c>
       <c r="G67">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="H67">
-        <v>793</v>
+        <v>1153</v>
       </c>
       <c r="I67">
-        <v>1060</v>
+        <v>1564</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B68">
         <v>1243</v>
       </c>
       <c r="C68">
-        <v>153</v>
+        <v>221</v>
       </c>
       <c r="D68">
         <v>6</v>
       </c>
       <c r="E68">
-        <v>159</v>
+        <v>227</v>
       </c>
       <c r="F68">
-        <v>331</v>
+        <v>538</v>
       </c>
       <c r="G68">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="H68">
-        <v>417</v>
+        <v>627</v>
       </c>
       <c r="I68">
-        <v>576</v>
+        <v>854</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B69">
         <v>2638</v>
       </c>
       <c r="C69">
-        <v>156</v>
+        <v>298</v>
       </c>
       <c r="D69">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E69">
-        <v>184</v>
+        <v>329</v>
       </c>
       <c r="F69">
-        <v>399</v>
+        <v>1019</v>
       </c>
       <c r="G69">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="H69">
-        <v>555</v>
+        <v>1179</v>
       </c>
       <c r="I69">
-        <v>739</v>
+        <v>1508</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="B70">
         <v>1860</v>
       </c>
       <c r="C70">
-        <v>88</v>
+        <v>169</v>
       </c>
       <c r="D70">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E70">
-        <v>102</v>
+        <v>185</v>
       </c>
       <c r="F70">
-        <v>264</v>
+        <v>744</v>
       </c>
       <c r="G70">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="H70">
-        <v>372</v>
+        <v>855</v>
       </c>
       <c r="I70">
-        <v>474</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="B71">
         <v>1640</v>
       </c>
       <c r="C71">
-        <v>94</v>
+        <v>215</v>
       </c>
       <c r="D71">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E71">
-        <v>98</v>
+        <v>224</v>
       </c>
       <c r="F71">
-        <v>215</v>
+        <v>547</v>
       </c>
       <c r="G71">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="H71">
-        <v>240</v>
+        <v>577</v>
       </c>
       <c r="I71">
-        <v>338</v>
+        <v>801</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="B72">
         <v>116695</v>
       </c>
       <c r="C72">
-        <v>9900</v>
+        <v>18128</v>
       </c>
       <c r="D72">
-        <v>888</v>
+        <v>1010</v>
       </c>
       <c r="E72">
-        <v>10788</v>
+        <v>19138</v>
       </c>
       <c r="F72">
-        <v>19607</v>
+        <v>41460</v>
       </c>
       <c r="G72">
-        <v>4889</v>
+        <v>5231</v>
       </c>
       <c r="H72">
-        <v>24496</v>
+        <v>46691</v>
       </c>
       <c r="I72">
-        <v>35284</v>
+        <v>65829</v>
       </c>
     </row>
   </sheetData>
@@ -3653,7 +3671,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="B1"/>
       <c r="C1"/>
@@ -3712,25 +3730,25 @@
         <v>2120</v>
       </c>
       <c r="C4">
-        <v>184</v>
+        <v>357</v>
       </c>
       <c r="D4">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E4">
-        <v>198</v>
+        <v>372</v>
       </c>
       <c r="F4">
-        <v>320</v>
+        <v>628</v>
       </c>
       <c r="G4">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="H4">
-        <v>361</v>
+        <v>676</v>
       </c>
       <c r="I4">
-        <v>559</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="5">
@@ -3741,25 +3759,25 @@
         <v>2258</v>
       </c>
       <c r="C5">
-        <v>187</v>
+        <v>318</v>
       </c>
       <c r="D5">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E5">
-        <v>205</v>
+        <v>340</v>
       </c>
       <c r="F5">
-        <v>313</v>
+        <v>695</v>
       </c>
       <c r="G5">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="H5">
-        <v>357</v>
+        <v>744</v>
       </c>
       <c r="I5">
-        <v>562</v>
+        <v>1084</v>
       </c>
     </row>
     <row r="6">
@@ -3770,25 +3788,25 @@
         <v>2060</v>
       </c>
       <c r="C6">
-        <v>255</v>
+        <v>422</v>
       </c>
       <c r="D6">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="E6">
-        <v>268</v>
+        <v>441</v>
       </c>
       <c r="F6">
-        <v>342</v>
+        <v>595</v>
       </c>
       <c r="G6">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="H6">
-        <v>383</v>
+        <v>644</v>
       </c>
       <c r="I6">
-        <v>651</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="7">
@@ -3799,25 +3817,25 @@
         <v>1790</v>
       </c>
       <c r="C7">
-        <v>275</v>
+        <v>401</v>
       </c>
       <c r="D7">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E7">
-        <v>300</v>
+        <v>429</v>
       </c>
       <c r="F7">
-        <v>352</v>
+        <v>584</v>
       </c>
       <c r="G7">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H7">
-        <v>430</v>
+        <v>663</v>
       </c>
       <c r="I7">
-        <v>730</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="8">
@@ -3828,25 +3846,25 @@
         <v>2482</v>
       </c>
       <c r="C8">
-        <v>277</v>
+        <v>463</v>
       </c>
       <c r="D8">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="E8">
-        <v>299</v>
+        <v>490</v>
       </c>
       <c r="F8">
-        <v>376</v>
+        <v>685</v>
       </c>
       <c r="G8">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H8">
-        <v>438</v>
+        <v>748</v>
       </c>
       <c r="I8">
-        <v>737</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="9">
@@ -3857,25 +3875,25 @@
         <v>2774</v>
       </c>
       <c r="C9">
-        <v>249</v>
+        <v>461</v>
       </c>
       <c r="D9">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="E9">
-        <v>283</v>
+        <v>501</v>
       </c>
       <c r="F9">
-        <v>473</v>
+        <v>906</v>
       </c>
       <c r="G9">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="H9">
-        <v>555</v>
+        <v>991</v>
       </c>
       <c r="I9">
-        <v>838</v>
+        <v>1492</v>
       </c>
     </row>
     <row r="10">
@@ -3886,25 +3904,25 @@
         <v>2693</v>
       </c>
       <c r="C10">
-        <v>282</v>
+        <v>475</v>
       </c>
       <c r="D10">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E10">
-        <v>310</v>
+        <v>504</v>
       </c>
       <c r="F10">
-        <v>392</v>
+        <v>722</v>
       </c>
       <c r="G10">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="H10">
-        <v>459</v>
+        <v>794</v>
       </c>
       <c r="I10">
-        <v>769</v>
+        <v>1298</v>
       </c>
     </row>
     <row r="11">
@@ -3915,25 +3933,25 @@
         <v>1664</v>
       </c>
       <c r="C11">
-        <v>169</v>
+        <v>263</v>
       </c>
       <c r="D11">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="E11">
-        <v>182</v>
+        <v>282</v>
       </c>
       <c r="F11">
-        <v>270</v>
+        <v>461</v>
       </c>
       <c r="G11">
-        <v>26</v>
+        <v>47</v>
       </c>
       <c r="H11">
-        <v>296</v>
+        <v>508</v>
       </c>
       <c r="I11">
-        <v>478</v>
+        <v>790</v>
       </c>
     </row>
     <row r="12">
@@ -3944,25 +3962,25 @@
         <v>2224</v>
       </c>
       <c r="C12">
-        <v>316</v>
+        <v>496</v>
       </c>
       <c r="D12">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="E12">
-        <v>330</v>
+        <v>514</v>
       </c>
       <c r="F12">
-        <v>365</v>
+        <v>664</v>
       </c>
       <c r="G12">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H12">
-        <v>401</v>
+        <v>704</v>
       </c>
       <c r="I12">
-        <v>731</v>
+        <v>1218</v>
       </c>
     </row>
     <row r="13">
@@ -3973,25 +3991,25 @@
         <v>1497</v>
       </c>
       <c r="C13">
-        <v>123</v>
+        <v>233</v>
       </c>
       <c r="D13">
         <v>19</v>
       </c>
       <c r="E13">
-        <v>142</v>
+        <v>252</v>
       </c>
       <c r="F13">
-        <v>264</v>
+        <v>518</v>
       </c>
       <c r="G13">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="H13">
-        <v>327</v>
+        <v>585</v>
       </c>
       <c r="I13">
-        <v>469</v>
+        <v>837</v>
       </c>
     </row>
     <row r="14">
@@ -4002,25 +4020,25 @@
         <v>2407</v>
       </c>
       <c r="C14">
-        <v>228</v>
+        <v>395</v>
       </c>
       <c r="D14">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="E14">
-        <v>251</v>
+        <v>424</v>
       </c>
       <c r="F14">
-        <v>479</v>
+        <v>878</v>
       </c>
       <c r="G14">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="H14">
-        <v>563</v>
+        <v>964</v>
       </c>
       <c r="I14">
-        <v>814</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="15">
@@ -4031,25 +4049,25 @@
         <v>3243</v>
       </c>
       <c r="C15">
-        <v>256</v>
+        <v>463</v>
       </c>
       <c r="D15">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="E15">
-        <v>305</v>
+        <v>518</v>
       </c>
       <c r="F15">
-        <v>374</v>
+        <v>871</v>
       </c>
       <c r="G15">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H15">
-        <v>488</v>
+        <v>993</v>
       </c>
       <c r="I15">
-        <v>793</v>
+        <v>1511</v>
       </c>
     </row>
     <row r="16">
@@ -4060,25 +4078,25 @@
         <v>2435</v>
       </c>
       <c r="C16">
-        <v>344</v>
+        <v>543</v>
       </c>
       <c r="D16">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E16">
-        <v>383</v>
+        <v>584</v>
       </c>
       <c r="F16">
-        <v>523</v>
+        <v>874</v>
       </c>
       <c r="G16">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H16">
-        <v>592</v>
+        <v>944</v>
       </c>
       <c r="I16">
-        <v>975</v>
+        <v>1528</v>
       </c>
     </row>
     <row r="17">
@@ -4089,25 +4107,25 @@
         <v>2799</v>
       </c>
       <c r="C17">
-        <v>251</v>
+        <v>563</v>
       </c>
       <c r="D17">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E17">
-        <v>258</v>
+        <v>575</v>
       </c>
       <c r="F17">
-        <v>367</v>
+        <v>848</v>
       </c>
       <c r="G17">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="H17">
-        <v>407</v>
+        <v>891</v>
       </c>
       <c r="I17">
-        <v>665</v>
+        <v>1466</v>
       </c>
     </row>
     <row r="18">
@@ -4118,25 +4136,25 @@
         <v>2252</v>
       </c>
       <c r="C18">
-        <v>235</v>
+        <v>431</v>
       </c>
       <c r="D18">
         <v>17</v>
       </c>
       <c r="E18">
-        <v>252</v>
+        <v>448</v>
       </c>
       <c r="F18">
-        <v>432</v>
+        <v>858</v>
       </c>
       <c r="G18">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="H18">
-        <v>478</v>
+        <v>908</v>
       </c>
       <c r="I18">
-        <v>730</v>
+        <v>1356</v>
       </c>
     </row>
     <row r="19">
@@ -4147,25 +4165,25 @@
         <v>1366</v>
       </c>
       <c r="C19">
-        <v>185</v>
+        <v>306</v>
       </c>
       <c r="D19">
         <v>6</v>
       </c>
       <c r="E19">
-        <v>191</v>
+        <v>312</v>
       </c>
       <c r="F19">
-        <v>297</v>
+        <v>532</v>
       </c>
       <c r="G19">
         <v>31</v>
       </c>
       <c r="H19">
-        <v>328</v>
+        <v>563</v>
       </c>
       <c r="I19">
-        <v>519</v>
+        <v>875</v>
       </c>
     </row>
     <row r="20">
@@ -4176,291 +4194,291 @@
         <v>1906</v>
       </c>
       <c r="C20">
-        <v>134</v>
+        <v>312</v>
       </c>
       <c r="D20">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="E20">
-        <v>136</v>
+        <v>329</v>
       </c>
       <c r="F20">
-        <v>236</v>
+        <v>647</v>
       </c>
       <c r="G20">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="H20">
-        <v>245</v>
+        <v>674</v>
       </c>
       <c r="I20">
-        <v>381</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B21">
         <v>35</v>
       </c>
       <c r="C21">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D21">
         <v>0</v>
       </c>
       <c r="E21">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F21">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="G21">
         <v>0</v>
       </c>
       <c r="H21">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="I21">
-        <v>0</v>
+        <v>22</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B22">
         <v>2937</v>
       </c>
       <c r="C22">
-        <v>258</v>
+        <v>504</v>
       </c>
       <c r="D22">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E22">
-        <v>281</v>
+        <v>529</v>
       </c>
       <c r="F22">
-        <v>508</v>
+        <v>1011</v>
       </c>
       <c r="G22">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="H22">
-        <v>599</v>
+        <v>1106</v>
       </c>
       <c r="I22">
-        <v>880</v>
+        <v>1635</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B23">
         <v>2055</v>
       </c>
       <c r="C23">
-        <v>148</v>
+        <v>278</v>
       </c>
       <c r="D23">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E23">
-        <v>168</v>
+        <v>299</v>
       </c>
       <c r="F23">
-        <v>350</v>
+        <v>705</v>
       </c>
       <c r="G23">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H23">
-        <v>426</v>
+        <v>782</v>
       </c>
       <c r="I23">
-        <v>594</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B24">
         <v>3096</v>
       </c>
       <c r="C24">
-        <v>231</v>
+        <v>500</v>
       </c>
       <c r="D24">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="E24">
-        <v>268</v>
+        <v>541</v>
       </c>
       <c r="F24">
-        <v>431</v>
+        <v>995</v>
       </c>
       <c r="G24">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="H24">
-        <v>524</v>
+        <v>1095</v>
       </c>
       <c r="I24">
-        <v>792</v>
+        <v>1636</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B25">
         <v>2122</v>
       </c>
       <c r="C25">
-        <v>278</v>
+        <v>482</v>
       </c>
       <c r="D25">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E25">
-        <v>302</v>
+        <v>508</v>
       </c>
       <c r="F25">
-        <v>459</v>
+        <v>825</v>
       </c>
       <c r="G25">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H25">
-        <v>557</v>
+        <v>927</v>
       </c>
       <c r="I25">
-        <v>859</v>
+        <v>1435</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B26">
         <v>2210</v>
       </c>
       <c r="C26">
-        <v>142</v>
+        <v>368</v>
       </c>
       <c r="D26">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E26">
-        <v>163</v>
+        <v>392</v>
       </c>
       <c r="F26">
-        <v>249</v>
+        <v>662</v>
       </c>
       <c r="G26">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="H26">
-        <v>297</v>
+        <v>714</v>
       </c>
       <c r="I26">
-        <v>460</v>
+        <v>1106</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B27">
         <v>2289</v>
       </c>
       <c r="C27">
-        <v>205</v>
+        <v>476</v>
       </c>
       <c r="D27">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E27">
-        <v>226</v>
+        <v>499</v>
       </c>
       <c r="F27">
-        <v>334</v>
+        <v>769</v>
       </c>
       <c r="G27">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="H27">
-        <v>385</v>
+        <v>825</v>
       </c>
       <c r="I27">
-        <v>611</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B28">
         <v>2649</v>
       </c>
       <c r="C28">
-        <v>205</v>
+        <v>490</v>
       </c>
       <c r="D28">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E28">
-        <v>252</v>
+        <v>543</v>
       </c>
       <c r="F28">
-        <v>340</v>
+        <v>778</v>
       </c>
       <c r="G28">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H28">
-        <v>458</v>
+        <v>897</v>
       </c>
       <c r="I28">
-        <v>710</v>
+        <v>1440</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B29">
         <v>3332</v>
       </c>
       <c r="C29">
-        <v>316</v>
+        <v>630</v>
       </c>
       <c r="D29">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="E29">
-        <v>363</v>
+        <v>684</v>
       </c>
       <c r="F29">
-        <v>675</v>
+        <v>1252</v>
       </c>
       <c r="G29">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="H29">
-        <v>809</v>
+        <v>1394</v>
       </c>
       <c r="I29">
-        <v>1172</v>
+        <v>2078</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B30">
         <v>5</v>
@@ -4475,45 +4493,45 @@
         <v>0</v>
       </c>
       <c r="F30">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G30">
         <v>0</v>
       </c>
       <c r="H30">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I30">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="B31">
         <v>58700</v>
       </c>
       <c r="C31">
-        <v>5733</v>
+        <v>10636</v>
       </c>
       <c r="D31">
-        <v>583</v>
+        <v>680</v>
       </c>
       <c r="E31">
-        <v>6316</v>
+        <v>11316</v>
       </c>
       <c r="F31">
-        <v>9521</v>
+        <v>18983</v>
       </c>
       <c r="G31">
-        <v>1642</v>
+        <v>1771</v>
       </c>
       <c r="H31">
-        <v>11163</v>
+        <v>20754</v>
       </c>
       <c r="I31">
-        <v>17479</v>
+        <v>32070</v>
       </c>
     </row>
   </sheetData>

</xml_diff>